<commit_message>
Revise MFT SDD: scope narrowed to the Boomi platform (Intelligrator & other programme projects removed). Add two platform pain points — no native CI/CD pipeline for MFT config (G-13) and no native enterprise password/secrets-manager path for MFT credentials (G-14). Diagram, Word, Excel, index.html updated; docs.zip rebuilt.
</commit_message>
<xml_diff>
--- a/assets/boomi-mft-sdd-capability-gap-register.xlsx
+++ b/assets/boomi-mft-sdd-capability-gap-register.xlsx
@@ -13,8 +13,8 @@
     <sheet name="Gap Register" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Capability Register'!$A$1:$F$16</definedName>
-    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">'Gap Register'!$A$1:$G$13</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Capability Register'!$A$1:$F$18</definedName>
+    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">'Gap Register'!$A$1:$G$15</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="169">
   <si>
     <t xml:space="preserve">MFT on Boomi (Thru) — Capability &amp; Gap Register</t>
   </si>
@@ -76,7 +76,7 @@
     <t xml:space="preserve">• Gap Register — limitations with impact, severity, and the mitigation/action each drives. Assign a named Owner and move Status from Open before build.</t>
   </si>
   <si>
-    <t xml:space="preserve">• High-severity gaps (residency/assurance and audit retention) are the two items that most affect go-live for OFFICIAL data.</t>
+    <t xml:space="preserve">• High-severity gaps (data residency/assurance, audit retention, and MFT credential/PAM sourcing) most affect go-live for OFFICIAL data. The missing native CI/CD pipeline (G-13) is the main delivery/operability drawback.</t>
   </si>
   <si>
     <t xml:space="preserve">• This register is the single source for the SDD Section 9 matrix and Section 11 gaps — keep them in step.</t>
@@ -313,6 +313,36 @@
     <t xml:space="preserve">Thru datasheet</t>
   </si>
   <si>
+    <t xml:space="preserve">C-16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Secrets Management Service</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Binds Integration runtime to cloud vaults (e.g. Azure Key Vault) for connector credentials; Nov-2025 release</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Runtime credentials — NOT confirmed for MFT endpoint/partner creds (see G-14)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Boomi community Nov-2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C-17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CI/CD via AtomSphere API + DevOps</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reference framework to promote Boomi assets through external DevOps tooling; not MFT-config-aware</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Config promotion must be built externally (see G-13)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Boomi DevOps guide</t>
+  </si>
+  <si>
     <t xml:space="preserve">Gap / limitation</t>
   </si>
   <si>
@@ -479,6 +509,30 @@
   </si>
   <si>
     <t xml:space="preserve">Deliberate re-configuration; sequence by risk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G-13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No native CI/CD pipeline for MFT config; promotion dev-&gt;test-&gt;prod is UI/admin-driven and environment-promotion not fully API-automatable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Manual promotion; weak traceability, review, rollback</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Build external CI/CD over AtomSphere APIs + DevOps tooling; hold config/routing table in Git; gated audited promotion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G-14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No documented native path to source MFT endpoint/partner credentials from enterprise password/secrets manager (e.g. CyberArk PAM); Secrets Mgmt Service targets Integration runtime + cloud vaults, not MFT partner creds</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Credentials in MFT store; weaker central rotation &amp; PAM governance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validate MFT credential sourcing with vendor; broker via Integration + secrets service or controlled vault sync; agree with Security</t>
   </si>
 </sst>
 </file>
@@ -674,76 +728,72 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="17">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="14" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1075,153 +1125,153 @@
   <dimension ref="A1:F22"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="3" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="3" style="0" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="6" t="n">
+      <c r="B5" s="5" t="n">
         <f aca="false">COUNTIF('Capability Register'!E:E,"GA")+COUNTIF('Capability Register'!E:E,"GA (legacy)")</f>
         <v>11</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="6" t="n">
+      <c r="B6" s="5" t="n">
         <f aca="false">COUNTIF('Capability Register'!E:E,"Confirm")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="6" t="n">
+      <c r="B7" s="5" t="n">
         <f aca="false">COUNTIF('Capability Register'!E:E,"Roadmap")</f>
         <v>1</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="6" t="n">
+      <c r="B8" s="5" t="n">
         <f aca="false">COUNTA('Capability Register'!A2:A100)</f>
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5" t="s">
+      <c r="A12" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B12" s="6" t="n">
+      <c r="B12" s="5" t="n">
         <f aca="false">COUNTIF('Gap Register'!D:D,"High")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5" t="s">
+      <c r="A13" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B13" s="6" t="n">
+      <c r="B13" s="5" t="n">
         <f aca="false">COUNTIF('Gap Register'!D:D,"Medium")</f>
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5" t="s">
+      <c r="A14" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="6" t="n">
+      <c r="B14" s="5" t="n">
         <f aca="false">COUNTIF('Gap Register'!D:D,"Low")</f>
         <v>2</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5" t="s">
+      <c r="A15" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B15" s="6" t="n">
+      <c r="B15" s="5" t="n">
         <f aca="false">COUNTA('Gap Register'!A2:A100)</f>
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7" t="s">
+      <c r="A18" s="6" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="8" t="s">
+      <c r="A19" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="B19" s="8"/>
-      <c r="C19" s="8"/>
-      <c r="D19" s="8"/>
-      <c r="E19" s="8"/>
-      <c r="F19" s="8"/>
+      <c r="B19" s="7"/>
+      <c r="C19" s="7"/>
+      <c r="D19" s="7"/>
+      <c r="E19" s="7"/>
+      <c r="F19" s="7"/>
     </row>
     <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="8" t="s">
+      <c r="A20" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="B20" s="8"/>
-      <c r="C20" s="8"/>
-      <c r="D20" s="8"/>
-      <c r="E20" s="8"/>
-      <c r="F20" s="8"/>
+      <c r="B20" s="7"/>
+      <c r="C20" s="7"/>
+      <c r="D20" s="7"/>
+      <c r="E20" s="7"/>
+      <c r="F20" s="7"/>
     </row>
     <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="8" t="s">
+      <c r="A21" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B21" s="8"/>
-      <c r="C21" s="8"/>
-      <c r="D21" s="8"/>
-      <c r="E21" s="8"/>
-      <c r="F21" s="8"/>
+      <c r="B21" s="7"/>
+      <c r="C21" s="7"/>
+      <c r="D21" s="7"/>
+      <c r="E21" s="7"/>
+      <c r="F21" s="7"/>
     </row>
     <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="8" t="s">
+      <c r="A22" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="B22" s="8"/>
-      <c r="C22" s="8"/>
-      <c r="D22" s="8"/>
-      <c r="E22" s="8"/>
-      <c r="F22" s="8"/>
+      <c r="B22" s="7"/>
+      <c r="C22" s="7"/>
+      <c r="D22" s="7"/>
+      <c r="E22" s="7"/>
+      <c r="F22" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -1245,339 +1295,379 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="20"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="B1" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="C1" s="9" t="s">
+      <c r="C1" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="E1" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="F1" s="8" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="B2" s="10" t="s">
+      <c r="B2" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="C2" s="10" t="s">
+      <c r="C2" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="D2" s="10" t="s">
+      <c r="D2" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="E2" s="11" t="s">
+      <c r="E2" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="F2" s="10" t="s">
+      <c r="F2" s="9" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="C3" s="12" t="s">
+      <c r="C3" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="D3" s="12" t="s">
+      <c r="D3" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="E3" s="13" t="s">
+      <c r="E3" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="F3" s="12" t="s">
+      <c r="F3" s="11" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="D4" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="E4" s="11" t="s">
+      <c r="E4" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="F4" s="10" t="s">
+      <c r="F4" s="9" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="B5" s="12" t="s">
+      <c r="B5" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="C5" s="12" t="s">
+      <c r="C5" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="D5" s="12" t="s">
+      <c r="D5" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="E5" s="14" t="s">
+      <c r="E5" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="F5" s="12" t="s">
+      <c r="F5" s="11" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="10" t="s">
+      <c r="A6" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C6" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="D6" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="E6" s="11" t="s">
+      <c r="E6" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="F6" s="10" t="s">
+      <c r="F6" s="9" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="12" t="s">
+      <c r="A7" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="B7" s="11" t="s">
         <v>52</v>
       </c>
-      <c r="C7" s="12" t="s">
+      <c r="C7" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="D7" s="12" t="s">
+      <c r="D7" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="E7" s="14" t="s">
+      <c r="E7" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="F7" s="12" t="s">
+      <c r="F7" s="11" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="C8" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="D8" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="E8" s="11" t="s">
+      <c r="E8" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="F8" s="10" t="s">
+      <c r="F8" s="9" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="12" t="s">
+      <c r="A9" s="11" t="s">
         <v>60</v>
       </c>
-      <c r="B9" s="12" t="s">
+      <c r="B9" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="C9" s="12" t="s">
+      <c r="C9" s="11" t="s">
         <v>62</v>
       </c>
-      <c r="D9" s="12" t="s">
+      <c r="D9" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="E9" s="14" t="s">
+      <c r="E9" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="F9" s="12" t="s">
+      <c r="F9" s="11" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="10" t="s">
+      <c r="A10" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C10" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="D10" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="E10" s="15" t="s">
+      <c r="E10" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="F10" s="10" t="s">
+      <c r="F10" s="9" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="12" t="s">
+      <c r="A11" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="B11" s="12" t="s">
+      <c r="B11" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="C11" s="12" t="s">
+      <c r="C11" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="D11" s="12" t="s">
+      <c r="D11" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="E11" s="14" t="s">
+      <c r="E11" s="13" t="s">
         <v>28</v>
       </c>
-      <c r="F11" s="12" t="s">
+      <c r="F11" s="11" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="10" t="s">
+      <c r="A12" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="C12" s="10" t="s">
+      <c r="C12" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="D12" s="10" t="s">
+      <c r="D12" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="E12" s="15" t="s">
+      <c r="E12" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="F12" s="10" t="s">
+      <c r="F12" s="9" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="12" t="s">
+      <c r="A13" s="11" t="s">
         <v>76</v>
       </c>
-      <c r="B13" s="12" t="s">
+      <c r="B13" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="C13" s="12" t="s">
+      <c r="C13" s="11" t="s">
         <v>78</v>
       </c>
-      <c r="D13" s="12" t="s">
+      <c r="D13" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="E13" s="14" t="s">
+      <c r="E13" s="13" t="s">
         <v>80</v>
       </c>
-      <c r="F13" s="12" t="s">
+      <c r="F13" s="11" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="10" t="s">
+      <c r="A14" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="B14" s="10" t="s">
+      <c r="B14" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="C14" s="10" t="s">
+      <c r="C14" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="D14" s="10" t="s">
+      <c r="D14" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="E14" s="11" t="s">
+      <c r="E14" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="F14" s="10" t="s">
+      <c r="F14" s="9" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="12" t="s">
+      <c r="A15" s="11" t="s">
         <v>85</v>
       </c>
-      <c r="B15" s="12" t="s">
+      <c r="B15" s="11" t="s">
         <v>86</v>
       </c>
-      <c r="C15" s="12" t="s">
+      <c r="C15" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="D15" s="12" t="s">
+      <c r="D15" s="11" t="s">
         <v>88</v>
       </c>
-      <c r="E15" s="16" t="s">
+      <c r="E15" s="15" t="s">
         <v>89</v>
       </c>
-      <c r="F15" s="12" t="s">
+      <c r="F15" s="11" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="10" t="s">
+      <c r="A16" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="B16" s="10" t="s">
+      <c r="B16" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="C16" s="10" t="s">
+      <c r="C16" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="D16" s="10" t="s">
+      <c r="D16" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="E16" s="11" t="s">
+      <c r="E16" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="F16" s="10" t="s">
+      <c r="F16" s="9" t="s">
         <v>94</v>
       </c>
     </row>
+    <row r="17" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="B17" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="C17" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="D17" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="E17" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="F17" s="11" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="9" t="s">
+        <v>100</v>
+      </c>
+      <c r="B18" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="C18" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="E18" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="F18" s="9" t="s">
+        <v>104</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F16"/>
+  <autoFilter ref="A1:F18"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -1594,318 +1684,364 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="10"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="9" t="s">
-        <v>95</v>
-      </c>
-      <c r="C1" s="9" t="s">
-        <v>96</v>
-      </c>
-      <c r="D1" s="9" t="s">
-        <v>97</v>
-      </c>
-      <c r="E1" s="9" t="s">
-        <v>98</v>
-      </c>
-      <c r="F1" s="9" t="s">
-        <v>99</v>
-      </c>
-      <c r="G1" s="9" t="s">
-        <v>100</v>
+      <c r="B1" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>108</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="10" t="s">
-        <v>101</v>
-      </c>
-      <c r="B2" s="10" t="s">
-        <v>102</v>
-      </c>
-      <c r="C2" s="10" t="s">
-        <v>103</v>
-      </c>
-      <c r="D2" s="15" t="s">
+      <c r="A2" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="D2" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="10" t="s">
-        <v>104</v>
-      </c>
-      <c r="F2" s="10" t="s">
-        <v>105</v>
-      </c>
-      <c r="G2" s="10" t="s">
-        <v>106</v>
+      <c r="E2" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="F2" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="G2" s="9" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="12" t="s">
-        <v>107</v>
-      </c>
-      <c r="B3" s="12" t="s">
-        <v>108</v>
-      </c>
-      <c r="C3" s="12" t="s">
-        <v>109</v>
-      </c>
-      <c r="D3" s="16" t="s">
+      <c r="A3" s="11" t="s">
+        <v>117</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="D3" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="12" t="s">
-        <v>110</v>
-      </c>
-      <c r="F3" s="12" t="s">
-        <v>105</v>
-      </c>
-      <c r="G3" s="12" t="s">
-        <v>106</v>
+      <c r="E3" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="F3" s="11" t="s">
+        <v>115</v>
+      </c>
+      <c r="G3" s="11" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="10" t="s">
-        <v>111</v>
-      </c>
-      <c r="B4" s="10" t="s">
-        <v>112</v>
-      </c>
-      <c r="C4" s="10" t="s">
-        <v>113</v>
-      </c>
-      <c r="D4" s="17" t="s">
+      <c r="A4" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>122</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>123</v>
+      </c>
+      <c r="D4" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="10" t="s">
-        <v>114</v>
-      </c>
-      <c r="F4" s="10" t="s">
-        <v>105</v>
-      </c>
-      <c r="G4" s="10" t="s">
-        <v>106</v>
+      <c r="E4" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="F4" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="G4" s="9" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="11" t="s">
+        <v>125</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>126</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>127</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="F5" s="11" t="s">
         <v>115</v>
       </c>
-      <c r="B5" s="12" t="s">
+      <c r="G5" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="C5" s="12" t="s">
-        <v>117</v>
-      </c>
-      <c r="D5" s="13" t="s">
+    </row>
+    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="D6" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="E5" s="12" t="s">
-        <v>118</v>
-      </c>
-      <c r="F5" s="12" t="s">
-        <v>105</v>
-      </c>
-      <c r="G5" s="12" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="10" t="s">
-        <v>119</v>
-      </c>
-      <c r="B6" s="10" t="s">
-        <v>120</v>
-      </c>
-      <c r="C6" s="10" t="s">
-        <v>121</v>
-      </c>
-      <c r="D6" s="15" t="s">
+      <c r="E6" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="F6" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="G6" s="9" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="11" t="s">
+        <v>133</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>134</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>135</v>
+      </c>
+      <c r="D7" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="E6" s="10" t="s">
-        <v>122</v>
-      </c>
-      <c r="F6" s="10" t="s">
-        <v>105</v>
-      </c>
-      <c r="G6" s="10" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="12" t="s">
-        <v>123</v>
-      </c>
-      <c r="B7" s="12" t="s">
-        <v>124</v>
-      </c>
-      <c r="C7" s="12" t="s">
-        <v>125</v>
-      </c>
-      <c r="D7" s="13" t="s">
+      <c r="E7" s="11" t="s">
+        <v>136</v>
+      </c>
+      <c r="F7" s="11" t="s">
+        <v>115</v>
+      </c>
+      <c r="G7" s="11" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>140</v>
+      </c>
+      <c r="F8" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="G8" s="9" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="11" t="s">
+        <v>141</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>142</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>143</v>
+      </c>
+      <c r="D9" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="E7" s="12" t="s">
-        <v>126</v>
-      </c>
-      <c r="F7" s="12" t="s">
-        <v>105</v>
-      </c>
-      <c r="G7" s="12" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="10" t="s">
-        <v>127</v>
-      </c>
-      <c r="B8" s="10" t="s">
-        <v>128</v>
-      </c>
-      <c r="C8" s="10" t="s">
-        <v>129</v>
-      </c>
-      <c r="D8" s="11" t="s">
+      <c r="E9" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="F9" s="11" t="s">
+        <v>115</v>
+      </c>
+      <c r="G9" s="11" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>146</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>147</v>
+      </c>
+      <c r="D10" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>148</v>
+      </c>
+      <c r="F10" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="G10" s="9" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="11" t="s">
+        <v>149</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="D11" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="E11" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="F11" s="11" t="s">
+        <v>115</v>
+      </c>
+      <c r="G11" s="11" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="D12" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="E8" s="10" t="s">
-        <v>130</v>
-      </c>
-      <c r="F8" s="10" t="s">
-        <v>105</v>
-      </c>
-      <c r="G8" s="10" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="12" t="s">
-        <v>131</v>
-      </c>
-      <c r="B9" s="12" t="s">
-        <v>132</v>
-      </c>
-      <c r="C9" s="12" t="s">
-        <v>133</v>
-      </c>
-      <c r="D9" s="13" t="s">
+      <c r="E12" s="9" t="s">
+        <v>156</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="G12" s="9" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>159</v>
+      </c>
+      <c r="D13" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="E9" s="12" t="s">
-        <v>134</v>
-      </c>
-      <c r="F9" s="12" t="s">
-        <v>105</v>
-      </c>
-      <c r="G9" s="12" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="10" t="s">
-        <v>135</v>
-      </c>
-      <c r="B10" s="10" t="s">
-        <v>136</v>
-      </c>
-      <c r="C10" s="10" t="s">
-        <v>137</v>
-      </c>
-      <c r="D10" s="15" t="s">
+      <c r="E13" s="11" t="s">
+        <v>160</v>
+      </c>
+      <c r="F13" s="11" t="s">
+        <v>115</v>
+      </c>
+      <c r="G13" s="11" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>162</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="D14" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="E10" s="10" t="s">
-        <v>138</v>
-      </c>
-      <c r="F10" s="10" t="s">
-        <v>105</v>
-      </c>
-      <c r="G10" s="10" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="12" t="s">
-        <v>139</v>
-      </c>
-      <c r="B11" s="12" t="s">
-        <v>140</v>
-      </c>
-      <c r="C11" s="12" t="s">
-        <v>141</v>
-      </c>
-      <c r="D11" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="E11" s="12" t="s">
-        <v>142</v>
-      </c>
-      <c r="F11" s="12" t="s">
-        <v>105</v>
-      </c>
-      <c r="G11" s="12" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="10" t="s">
-        <v>143</v>
-      </c>
-      <c r="B12" s="10" t="s">
-        <v>144</v>
-      </c>
-      <c r="C12" s="10" t="s">
-        <v>145</v>
-      </c>
-      <c r="D12" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="E12" s="10" t="s">
-        <v>146</v>
-      </c>
-      <c r="F12" s="10" t="s">
-        <v>105</v>
-      </c>
-      <c r="G12" s="10" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="12" t="s">
-        <v>147</v>
-      </c>
-      <c r="B13" s="12" t="s">
-        <v>148</v>
-      </c>
-      <c r="C13" s="12" t="s">
-        <v>149</v>
-      </c>
-      <c r="D13" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="E13" s="12" t="s">
-        <v>150</v>
-      </c>
-      <c r="F13" s="12" t="s">
-        <v>105</v>
-      </c>
-      <c r="G13" s="12" t="s">
-        <v>106</v>
+      <c r="E14" s="9" t="s">
+        <v>164</v>
+      </c>
+      <c r="F14" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="G14" s="9" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>166</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>167</v>
+      </c>
+      <c r="D15" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="E15" s="11" t="s">
+        <v>168</v>
+      </c>
+      <c r="F15" s="11" t="s">
+        <v>115</v>
+      </c>
+      <c r="G15" s="11" t="s">
+        <v>116</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G13"/>
+  <autoFilter ref="A1:G15"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
Show MFT integrated with the Integration & API-management platform. Fig 1 enriched (API Control Plane, Developer Portal, Integration Flow Designer/Runtime, Cloud API Management, external/internal API gateways, Kong) with the Boomi MFT Connector bridging integration flows to the config-driven MFT engine; API-executions vs config/deploy channels. New Fig 2: MFT<->Integration Platform connector mechanism (control vs data channels, direct file exchange, orchestration/reporting). Word/Excel/HTML updated; docs.zip rebuilt.
</commit_message>
<xml_diff>
--- a/assets/boomi-mft-sdd-capability-gap-register.xlsx
+++ b/assets/boomi-mft-sdd-capability-gap-register.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Gap Register" sheetId="3" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Capability Register'!$A$1:$F$18</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Capability Register'!$A$1:$F$20</definedName>
     <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">'Gap Register'!$A$1:$G$15</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="179">
   <si>
     <t xml:space="preserve">MFT on Boomi (Thru) — Capability &amp; Gap Register</t>
   </si>
@@ -341,6 +341,36 @@
   </si>
   <si>
     <t xml:space="preserve">Boomi DevOps guide</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C-18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Integration Platform interoperability</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Boomi MFT Connector lets an integration process invoke MFT file-transfer flows (event-driven orchestration; control vs data channels)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MFT triggered/orchestrated by integration flows; one platform &amp; audit trail</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Boomi MFT connector docs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C-19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">API Management fronting MFT/integration APIs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAM + external/internal API gateways (and Kong) publish and secure MFT/integration APIs to consumers and HoD apps</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Governed API access instead of point-to-point</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Boomi CAM docs</t>
   </si>
   <si>
     <t xml:space="preserve">Gap / limitation</t>
@@ -1154,7 +1184,7 @@
       </c>
       <c r="B5" s="5" t="n">
         <f aca="false">COUNTIF('Capability Register'!E:E,"GA")+COUNTIF('Capability Register'!E:E,"GA (legacy)")</f>
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1163,7 +1193,7 @@
       </c>
       <c r="B6" s="5" t="n">
         <f aca="false">COUNTIF('Capability Register'!E:E,"Confirm")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1181,7 +1211,7 @@
       </c>
       <c r="B8" s="5" t="n">
         <f aca="false">COUNTA('Capability Register'!A2:A100)</f>
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1295,7 +1325,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
@@ -1666,8 +1696,48 @@
         <v>104</v>
       </c>
     </row>
+    <row r="19" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="11" t="s">
+        <v>105</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="C19" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="D19" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="E19" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="F19" s="11" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="B20" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="C20" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="E20" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="F20" s="9" t="s">
+        <v>114</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F18"/>
+  <autoFilter ref="A1:F20"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -1700,344 +1770,344 @@
         <v>18</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>105</v>
+        <v>115</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>108</v>
+        <v>118</v>
       </c>
       <c r="F1" s="8" t="s">
-        <v>109</v>
+        <v>119</v>
       </c>
       <c r="G1" s="8" t="s">
-        <v>110</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="s">
-        <v>111</v>
+        <v>121</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>112</v>
+        <v>122</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="D2" s="14" t="s">
         <v>10</v>
       </c>
       <c r="E2" s="9" t="s">
-        <v>114</v>
+        <v>124</v>
       </c>
       <c r="F2" s="9" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="G2" s="9" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="11" t="s">
-        <v>117</v>
+        <v>127</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>119</v>
+        <v>129</v>
       </c>
       <c r="D3" s="15" t="s">
         <v>9</v>
       </c>
       <c r="E3" s="11" t="s">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="F3" s="11" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="G3" s="11" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>121</v>
+        <v>131</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>122</v>
+        <v>132</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>123</v>
+        <v>133</v>
       </c>
       <c r="D4" s="16" t="s">
         <v>9</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>124</v>
+        <v>134</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="11" t="s">
-        <v>125</v>
+        <v>135</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>126</v>
+        <v>136</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>127</v>
+        <v>137</v>
       </c>
       <c r="D5" s="12" t="s">
         <v>10</v>
       </c>
       <c r="E5" s="11" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="G5" s="11" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>129</v>
+        <v>139</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>130</v>
+        <v>140</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>131</v>
+        <v>141</v>
       </c>
       <c r="D6" s="14" t="s">
         <v>10</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="G6" s="9" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="11" t="s">
-        <v>133</v>
+        <v>143</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>134</v>
+        <v>144</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>135</v>
+        <v>145</v>
       </c>
       <c r="D7" s="12" t="s">
         <v>10</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>136</v>
+        <v>146</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="G7" s="11" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="9" t="s">
-        <v>137</v>
+        <v>147</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>138</v>
+        <v>148</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>139</v>
+        <v>149</v>
       </c>
       <c r="D8" s="10" t="s">
         <v>11</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>140</v>
+        <v>150</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="G8" s="9" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="11" t="s">
-        <v>141</v>
+        <v>151</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>142</v>
+        <v>152</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>143</v>
+        <v>153</v>
       </c>
       <c r="D9" s="12" t="s">
         <v>10</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>144</v>
+        <v>154</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="G9" s="11" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="9" t="s">
-        <v>145</v>
+        <v>155</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>146</v>
+        <v>156</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>147</v>
+        <v>157</v>
       </c>
       <c r="D10" s="14" t="s">
         <v>10</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>148</v>
+        <v>158</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="G10" s="9" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="s">
-        <v>149</v>
+        <v>159</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>150</v>
+        <v>160</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>151</v>
+        <v>161</v>
       </c>
       <c r="D11" s="12" t="s">
         <v>10</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>152</v>
+        <v>162</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="G11" s="11" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="9" t="s">
-        <v>153</v>
+        <v>163</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>154</v>
+        <v>164</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>155</v>
+        <v>165</v>
       </c>
       <c r="D12" s="10" t="s">
         <v>11</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>156</v>
+        <v>166</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="G12" s="9" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
-        <v>157</v>
+        <v>167</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>158</v>
+        <v>168</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="D13" s="12" t="s">
         <v>10</v>
       </c>
       <c r="E13" s="11" t="s">
-        <v>160</v>
+        <v>170</v>
       </c>
       <c r="F13" s="11" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="G13" s="11" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="s">
-        <v>161</v>
+        <v>171</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>162</v>
+        <v>172</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>163</v>
+        <v>173</v>
       </c>
       <c r="D14" s="14" t="s">
         <v>10</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>164</v>
+        <v>174</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="G14" s="9" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>165</v>
+        <v>175</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>166</v>
+        <v>176</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>167</v>
+        <v>177</v>
       </c>
       <c r="D15" s="15" t="s">
         <v>9</v>
       </c>
       <c r="E15" s="11" t="s">
-        <v>168</v>
+        <v>178</v>
       </c>
       <c r="F15" s="11" t="s">
-        <v>115</v>
+        <v>125</v>
       </c>
       <c r="G15" s="11" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
     </row>
   </sheetData>

</xml_diff>